<commit_message>
Refactor CSV tables for consistency and accuracy
- Updated the order of columns in 01_missing_values_breakdown.csv for better readability.
- Corrected the order of subjects in 24_bangladesh_top_subjects.csv.
- Moved University of Minnesota Libraries Publishing to the correct position in 25_bangladesh_top_publishers.csv.
- Adjusted the order of foreign collaboration partners in 27_bangladesh_foreign_collaboration_partners.csv.
- Fixed the list of top repeat authors in 28_bangladesh_top_repeat_authors.csv by correcting author names and counts.
- Updated all_retraction_watch_eda_tables.xlsx to reflect recent changes.
</commit_message>
<xml_diff>
--- a/tables/all_retraction_watch_eda_tables.xlsx
+++ b/tables/all_retraction_watch_eda_tables.xlsx
@@ -1,40 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing_Values" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duplication_Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning_Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engineered_Stats" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delay_Quantiles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual_Trends" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retraction_Matrix" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort_Lag_Counts" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top15_Reasons" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top15_Countries" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top15_Publishing_Nations" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Highest_Rate_Nations" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top10_Publishers" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top10_Journals" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paid_vs_OpenAccess" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paid_Lag_Pct" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Baseline_Metrics" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Annual_vs_Global" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Top_Universities" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Top_Reasons" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_vs_Global_Reasons" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_vs_Global_Lag" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Top_Subjects" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Top_Publishers" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Foreign_Partners" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Repeat_Authors" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Top_Journals" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD_Sector_Breakdown" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Missing_Values" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Duplication_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cleaning_Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Engineered_Stats" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Delay_Quantiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Annual_Trends" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Retraction_Matrix" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cohort_Lag_Counts" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Top15_Reasons" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Top15_Countries" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Top15_Publishing_Nations" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Highest_Rate_Nations" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Top10_Publishers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Top10_Journals" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Paid_vs_OpenAccess" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Paid_Lag_Pct" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="BD_Baseline_Metrics" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="BD_Annual_vs_Global" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="BD_Top_Universities" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="BD_Top_Reasons" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="BD_vs_Global_Reasons" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="BD_vs_Global_Lag" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="BD_Top_Subjects" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="BD_Top_Publishers" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="BD_Foreign_Partners" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="BD_Repeat_Authors" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="BD_Top_Journals" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="BD_Sector_Breakdown" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,16 +44,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -64,7 +61,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -72,21 +69,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,17 +444,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Missing Count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Missing Percentage (%)</t>
         </is>
@@ -566,7 +554,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Paywalled</t>
+          <t>Record ID</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -579,7 +567,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Subject</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -592,7 +580,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RetractionNature</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -605,7 +593,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OriginalPaperDate</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -618,7 +606,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Record ID</t>
+          <t>Publisher</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -631,7 +619,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>RetractionDate</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -657,7 +645,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -670,7 +658,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Author</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -683,7 +671,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Publisher</t>
+          <t>OriginalPaperDate</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -696,7 +684,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>RetractionNature</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -709,7 +697,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Subject</t>
+          <t>Reason</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -722,7 +710,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RetractionDate</t>
+          <t>Paywalled</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -747,12 +735,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -923,62 +911,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Citable documents</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Citations</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Self-citations</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Citations per document</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>H index</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Retracted_Papers</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Retraction_Rate_%</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Retractions_per_10k</t>
         </is>
@@ -1629,67 +1617,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Citable documents</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Citations</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Self-citations</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Citations per document</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>H index</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Retracted_Papers</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Retraction_Rate_%</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Retractions_per_10k</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Rate_Rank</t>
         </is>
@@ -2790,12 +2778,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Publisher</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -2916,12 +2904,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -3042,27 +3030,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Paywalled</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Paper_Count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Median_Delay_Years</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Mean_Delay_Years</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Pct_Retracted_Under_1yr</t>
         </is>
@@ -3121,27 +3109,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Paywalled</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>&lt; 1 Year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>1 to 3 Years</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>3 to 5 Years</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>&gt; 5 Years</t>
         </is>
@@ -3200,12 +3188,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -3322,22 +3310,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Global_Retractions</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>BD_Retractions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>BD_Share_of_Global_%</t>
         </is>
@@ -3736,12 +3724,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>University</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -3882,17 +3870,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Duplication Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Duplicate Count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Percentage (%)</t>
         </is>
@@ -3965,12 +3953,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Occurrence_Count</t>
         </is>
@@ -4111,22 +4099,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Bangladesh (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Global (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Difference (BD - Global)</t>
         </is>
@@ -4291,17 +4279,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Percentage (%)</t>
         </is>
@@ -4442,12 +4430,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -4516,7 +4504,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(HSC) Medicine - General</t>
+          <t>(HSC) Medicine - Infectious Disease</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4526,7 +4514,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>(HSC) Medicine - Infectious Disease</t>
+          <t>(HSC) Medicine - General</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4568,12 +4556,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Publisher</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -4662,7 +4650,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>University of Minnesota Libraries Publishing</t>
+          <t>MDPI</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4672,7 +4660,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MDPI</t>
+          <t>University of Minnesota Libraries Publishing</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4694,12 +4682,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Foreign_Country</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Co_Affiliated_Retractions</t>
         </is>
@@ -4808,7 +4796,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4818,7 +4806,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4840,12 +4828,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Author_Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -4914,7 +4902,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A K Mohiuddin</t>
+          <t>Md Rezaul Islam</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4934,7 +4922,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tahia Tazin</t>
+          <t>Sami Bourouis</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4944,7 +4932,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sami Bourouis</t>
+          <t>Tahia Tazin</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4954,7 +4942,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Md Rezaul Islam</t>
+          <t>A K Mohiuddin</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4964,7 +4952,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fahadul Islam</t>
+          <t>Abu Reza Md Towfiqul Islam</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4986,12 +4974,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retraction_Count</t>
         </is>
@@ -5112,12 +5100,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Paper_Count</t>
         </is>
@@ -5178,12 +5166,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Remediation Step</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -5244,27 +5232,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time_To_Retraction_Days</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Time_To_Retraction_Years</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>RetractionYear</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>OriginalYear</t>
         </is>
@@ -5437,12 +5425,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -5571,17 +5559,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Retractions_Executed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Original_Papers_Published</t>
         </is>
@@ -5954,54 +5942,54 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>OriginalYear</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n">
+      <c r="B1" t="n">
         <v>2012</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" t="n">
         <v>2013</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" t="n">
         <v>2014</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" t="n">
         <v>2015</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" t="n">
         <v>2016</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" t="n">
         <v>2017</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" t="n">
         <v>2018</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" t="n">
         <v>2019</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" t="n">
         <v>2020</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" t="n">
         <v>2021</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" t="n">
         <v>2022</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" t="n">
         <v>2023</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" t="n">
         <v>2024</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" t="n">
         <v>2025</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -6720,27 +6708,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>OriginalYear</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>&lt; 1 Year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>1 to 3 Years</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>3 to 5 Years</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>&gt; 5 Years</t>
         </is>
@@ -6982,12 +6970,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Occurrence_Count</t>
         </is>

</xml_diff>